<commit_message>
Site updated: 2026-09-29 09:15:10
</commit_message>
<xml_diff>
--- a/table/WILB.xlsx
+++ b/table/WILB.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1megalovania\阴间\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1megalovania\Hexo-Blog\source\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D7EDA12-B3B0-499F-99B6-B2CF8E802E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42E5378-2DEF-492E-B866-D8B39DB5ADB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="21806" windowHeight="13886" xr2:uid="{5C47B7C5-F1A9-4074-9C02-D87063408508}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="153">
   <si>
     <t>最喜欢的数字</t>
   </si>
@@ -511,6 +511,53 @@
   </si>
   <si>
     <t>刚上高中计划选科物化生，于是起初没有认真学地理。因为第一次测验成绩很差被地理老师叫去在试卷上写了详细的解题过程后，开始沉迷于给每道地理题写详解。曾取得过全区期末成绩地理第48名。是高考时得分率最高的科目。因为方向感很好所以即使不在应试环境下地理一直也算我的优势。</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>最喜欢的调味品</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>芥末</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>优先考虑级</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>较喜欢级</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>醋</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>不知为何，像是别人不会像我一样生啃柠檬一样地、我莫名地很能吃得下去芥末。第一次去吃滨寿司的时候尝试了一下，从此以后我的寿司蘸料只剩下了芥末。冲脑袋但是不会激得我起痘，甚至有种清新感，对我来说是辣椒的绝对上位。将来果然是想要把芥末生腌柠檬片定作我的常用开胃菜。</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>最喜欢的糕点</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>老婆饼</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>能把糖做成这样软度适中又恰好在我的甜度接受范围内的内馅的人简直是天才。</t>
+  </si>
+  <si>
+    <t>最喜欢的面包品种</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>可颂</t>
+    <phoneticPr fontId="19" type="noConversion"/>
+  </si>
+  <si>
+    <t>面包对我来说我都喜欢。选择可颂是因为喜欢它的中文名字。若是要给我自己设计一款面包绝对得是可颂啊。</t>
     <phoneticPr fontId="19" type="noConversion"/>
   </si>
 </sst>
@@ -1549,7 +1596,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FB6DA0B-1B05-4DE3-A377-1934D96B2412}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr defaultRowHeight="15.9" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.2109375" style="2" bestFit="1" customWidth="1"/>
@@ -2197,6 +2244,51 @@
         <v>131</v>
       </c>
     </row>
+    <row r="42" spans="1:5" ht="95.15" x14ac:dyDescent="0.35">
+      <c r="A42" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="31.75" x14ac:dyDescent="0.35">
+      <c r="A43" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="47.6" x14ac:dyDescent="0.35">
+      <c r="A44" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>